<commit_message>
Add audit tooling (ESLint gate, husky, CI), AUDIT.md, codemod; clean LaundroMat dead code
</commit_message>
<xml_diff>
--- a/audit/Audit-tool-by-tool.xlsx
+++ b/audit/Audit-tool-by-tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/SRsr/Desktop/deftbrain/audit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07FD0B7-60B3-E641-B4AD-4B7C8FF3CAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53D308B-E9DB-7B41-834D-4080550029AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" xr2:uid="{FC317A6B-1ECF-2545-8464-105F4E136AA9}"/>
   </bookViews>
@@ -1438,9 +1438,12 @@
         <v>126</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>127</v>
+      </c>
+      <c r="B129" s="1">
+        <v>46175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>